<commit_message>
Update lint review workflow and waiver artifacts
</commit_message>
<xml_diff>
--- a/LINT/outputs/lint_review.xlsx
+++ b/LINT/outputs/lint_review.xlsx
@@ -262,47 +262,165 @@
 waived: the issue comes from report_lint.waived</t>
       </text>
     </comment>
+    <comment ref="M2" authorId="0">
+      <text>
+        <t xml:space="preserve">Primary waiver rule shared by 32 issues.
+Shared issue IDs: DeadCode-ML_e84cae0edf25, DeadCode-ML_7fbcfb987ea2, DeadCode-ML_4061be3b213d, DeadCode-ML_37ccad7cafff, DeadCode-ML_5355615cf12e, DeadCode-ML_f4b3854a503a, DeadCode-ML_515337bfea90, DeadCode-ML_097ffa5f22ec, DeadCode-ML_51ab66d6b498, DeadCode-ML_14a921a01cb4, DeadCode-ML_6817476ffd8b, DeadCode-ML_1763cba8fabb, DeadCode-ML_4eb385741c5b, DeadCode-ML_fcc27bcb35f3, DeadCode-ML_9f84acebc779, DeadCode-ML_320417ba96fc, DeadCode-ML_8a1be6df56cf, DeadCode-ML_3f40c134f801, DeadCode-ML_520b0d4a7048, DeadCode-ML_fbb63c7ca9b7, DeadCode-ML_164f1d6db727, DeadCode-ML_323fbdc90de8, DeadCode-ML_75c765148170, DeadCode-ML_989754a375df, DeadCode-ML_c811eb95211b, DeadCode-ML_a870b15ab72f, DeadCode-ML_e22b6a54e417, DeadCode-ML_28eef1dad7ca, DeadCode-ML_366797be4f73, DeadCode-ML_c2740f9a65ca, DeadCode-ML_d48f18b9af6a</t>
+      </text>
+    </comment>
+    <comment ref="M3" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
     <comment ref="M4" authorId="0">
       <text>
-        <t xml:space="preserve">Primary waiver rule shared by 4 issues.
-Shared issue IDs: DeadCode-ML_4061be3b213d, DeadCode-ML_37ccad7cafff, DeadCode-ML_5355615cf12e</t>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
       </text>
     </comment>
     <comment ref="M5" authorId="0">
       <text>
-        <t xml:space="preserve">Shares waiver rule DeadCode-ML_741 with primary issue DeadCode-ML_7fbcfb987ea2.</t>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
       </text>
     </comment>
     <comment ref="M6" authorId="0">
       <text>
-        <t xml:space="preserve">Shares waiver rule DeadCode-ML_741 with primary issue DeadCode-ML_7fbcfb987ea2.</t>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
       </text>
     </comment>
     <comment ref="M7" authorId="0">
       <text>
-        <t xml:space="preserve">Shares waiver rule DeadCode-ML_741 with primary issue DeadCode-ML_7fbcfb987ea2.</t>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M8" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M9" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M10" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
       </text>
     </comment>
     <comment ref="M11" authorId="0">
       <text>
-        <t xml:space="preserve">Primary waiver rule shared by 2 issues.
-Shared issue IDs: DeadCode-ML_14a921a01cb4</t>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
       </text>
     </comment>
     <comment ref="M12" authorId="0">
       <text>
-        <t xml:space="preserve">Shares waiver rule DeadCode-ML_748 with primary issue DeadCode-ML_51ab66d6b498.</t>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M13" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M14" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M15" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M16" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M17" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M18" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M19" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M20" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M21" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M22" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M23" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M24" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M25" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M26" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M27" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M28" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M29" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
       </text>
     </comment>
     <comment ref="M30" authorId="0">
       <text>
-        <t xml:space="preserve">Primary waiver rule shared by 2 issues.
-Shared issue IDs: DeadCode-ML_366797be4f73</t>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
       </text>
     </comment>
     <comment ref="M31" authorId="0">
       <text>
-        <t xml:space="preserve">Shares waiver rule DeadCode-ML_767 with primary issue DeadCode-ML_28eef1dad7ca.</t>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M32" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
+      </text>
+    </comment>
+    <comment ref="M33" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule DeadCode-ML_739 with primary issue DeadCode-ML_3a66f0d939c6.</t>
       </text>
     </comment>
   </commentList>
@@ -548,48 +666,285 @@
 waived: the issue comes from report_lint.waived</t>
       </text>
     </comment>
+    <comment ref="M2" authorId="0">
+      <text>
+        <t xml:space="preserve">Primary waiver rule shared by 56 issues.
+Shared issue IDs: W164a_fd6a370a79ab, W164a_d93541370b31, W164a_7660b53e6188, W164a_c90a63b2d9e8, W164a_1d457f0d51fe, W164a_c078e63cfa3e, W164a_b1c30aa3f537, W164a_b16c35b5e10c, W164a_017526ab4c3d, W164a_c505e9870872, W164a_14c860086292, W164a_411e166bb6e8, W164a_97e34627177b, W164a_b105ea5a36d7, W164a_af9f5f624f8c, W164a_1064ea20e23f, W164a_f303846eddbf, W164a_1ab2b57028bc, W164a_d33034023f51, W164a_8efcf1475d55, W164a_043a813ca8f6, W164a_72d36f1914f2, W164a_e97c355c8578, W164a_8ae0b89979a0, W164a_4f28e5ce8f80, W164a_2cf4a06f09c5, W164a_5e0b6dc4ac33, W164a_4e84e698ed3e, W164a_a0c63c9da2e6, W164a_6fc4541b3f0d, W164a_453183e95577, W164a_4a2e5e0663a5, W164a_6ff437a3ada4, W164a_161793cb7dad, W164a_ebd65b48e89f, W164a_dc52da86c0c0, W164a_6fda0611280a, W164a_ea91e32f9aa7, W164a_ccf02468d9ed, W164a_6baf6e5ad83d, W164a_ad7c6281ae5d, W164a_4f36dd084a7e, W164a_fcad9e726414, W164a_f08d25377633, W164a_fe2225ff642e, W164a_33135cff7657, W164a_d681159d5355, W164a_d4ea1a544292, W164a_911d84fd734b, W164a_c236385e4a5a, W164a_87f654826bb3, W164a_f0e03f5a7b78, W164a_25c7ecc3014c, W164a_f4629a2c0a13, W164a_40e2f3cc3783</t>
+      </text>
+    </comment>
+    <comment ref="M3" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M4" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M5" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M6" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
     <comment ref="M7" authorId="0">
       <text>
-        <t xml:space="preserve">Primary waiver rule shared by 2 issues.
-Shared issue IDs: W164a_c078e63cfa3e</t>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
       </text>
     </comment>
     <comment ref="M8" authorId="0">
       <text>
-        <t xml:space="preserve">Shares waiver rule W164a_811 with primary issue W164a_1d457f0d51fe.</t>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M9" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M10" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M11" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M12" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
       </text>
     </comment>
     <comment ref="M13" authorId="0">
       <text>
-        <t xml:space="preserve">Primary waiver rule shared by 2 issues.
-Shared issue IDs: W164a_411e166bb6e8</t>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
       </text>
     </comment>
     <comment ref="M14" authorId="0">
       <text>
-        <t xml:space="preserve">Shares waiver rule W164a_791 with primary issue W164a_14c860086292.</t>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
       </text>
     </comment>
     <comment ref="M15" authorId="0">
       <text>
-        <t xml:space="preserve">Primary waiver rule shared by 2 issues.
-Shared issue IDs: W164a_b105ea5a36d7</t>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
       </text>
     </comment>
     <comment ref="M16" authorId="0">
       <text>
-        <t xml:space="preserve">Shares waiver rule W164a_793 with primary issue W164a_97e34627177b.</t>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M17" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M18" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
       </text>
     </comment>
     <comment ref="M19" authorId="0">
       <text>
-        <t xml:space="preserve">Primary waiver rule shared by 2 issues.
-Shared issue IDs: W164a_1ab2b57028bc</t>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
       </text>
     </comment>
     <comment ref="M20" authorId="0">
       <text>
-        <t xml:space="preserve">Shares waiver rule W164a_785 with primary issue W164a_f303846eddbf.</t>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M21" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M22" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M23" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M24" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M25" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M26" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M27" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M28" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M29" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M30" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M31" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M32" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M33" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M34" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M35" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M36" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M37" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M38" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M39" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M40" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M41" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M42" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M43" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M44" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M45" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M46" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M47" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M48" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M49" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M50" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M51" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M52" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M53" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M54" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M55" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M56" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
+      </text>
+    </comment>
+    <comment ref="M57" authorId="0">
+      <text>
+        <t xml:space="preserve">Shares waiver rule W164a_808 with primary issue W164a_aa9901c77213.</t>
       </text>
     </comment>
   </commentList>
@@ -18452,7 +18807,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Goal, Module, LineNumber, Statement, NodeType, PropertyList:LintPropertyName=Property_142</t>
+          <t xml:space="preserve">Goal</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -18502,7 +18857,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve">22-06-2026 13:10:10</t>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -18814,12 +19169,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -18864,12 +19219,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -18946,12 +19301,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -18986,7 +19341,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_740</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -18996,12 +19351,12 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -19078,12 +19433,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -19118,7 +19473,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_741</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -19128,12 +19483,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -19210,12 +19565,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -19250,7 +19605,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_741</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -19260,12 +19615,12 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -19342,12 +19697,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -19382,7 +19737,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_741</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -19392,12 +19747,12 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -19474,12 +19829,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -19514,7 +19869,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_741</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -19524,12 +19879,12 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -19606,12 +19961,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -19646,7 +20001,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_745</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -19656,12 +20011,12 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -19738,12 +20093,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -19778,7 +20133,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_746</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -19788,12 +20143,12 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -19870,12 +20225,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -19910,7 +20265,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_747</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -19920,12 +20275,12 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -20002,12 +20357,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -20042,7 +20397,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_748</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -20052,12 +20407,12 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -20134,12 +20489,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -20174,7 +20529,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_748</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -20184,12 +20539,12 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -20266,12 +20621,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -20306,7 +20661,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_750</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -20316,12 +20671,12 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -20398,12 +20753,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -20438,7 +20793,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_763</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -20448,12 +20803,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -20530,12 +20885,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -20570,7 +20925,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_764</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -20580,12 +20935,12 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -20662,12 +21017,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -20702,7 +21057,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_765</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -20712,12 +21067,12 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -20794,12 +21149,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -20834,7 +21189,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_766</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -20844,12 +21199,12 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -20926,12 +21281,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -20966,7 +21321,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_751</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -20976,12 +21331,12 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -21058,12 +21413,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -21098,7 +21453,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_752</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -21108,12 +21463,12 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -21190,12 +21545,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -21230,7 +21585,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_753</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -21240,12 +21595,12 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -21322,12 +21677,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -21362,7 +21717,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_754</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -21372,12 +21727,12 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -21454,12 +21809,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -21494,7 +21849,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_755</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -21504,12 +21859,12 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -21586,12 +21941,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -21626,7 +21981,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_756</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -21636,12 +21991,12 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -21718,12 +22073,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -21758,7 +22113,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_757</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -21768,12 +22123,12 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -21850,12 +22205,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -21890,7 +22245,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_758</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -21900,12 +22255,12 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -21982,12 +22337,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -22022,7 +22377,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_759</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -22032,12 +22387,12 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -22114,12 +22469,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -22154,7 +22509,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_760</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -22164,12 +22519,12 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -22246,12 +22601,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -22286,7 +22641,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_761</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -22296,12 +22651,12 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -22378,12 +22733,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -22418,7 +22773,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_762</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -22428,12 +22783,12 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -22510,12 +22865,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -22550,7 +22905,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_767</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -22560,12 +22915,12 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -22642,12 +22997,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -22682,7 +23037,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_767</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -22692,12 +23047,12 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -22774,12 +23129,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -22814,7 +23169,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_769</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -22824,12 +23179,12 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -22906,12 +23261,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_DATAGEN</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -22946,7 +23301,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t xml:space="preserve">DeadCode-ML_770</t>
+          <t xml:space="preserve">DeadCode-ML_739</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -22956,12 +23311,12 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -25745,12 +26100,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -25795,12 +26150,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -25902,12 +26257,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -25942,7 +26297,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_809</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -25952,12 +26307,12 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -26059,12 +26414,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -26099,7 +26454,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_814</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -26109,12 +26464,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -26216,12 +26571,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -26256,7 +26611,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_810</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -26266,12 +26621,12 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -26373,12 +26728,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -26413,7 +26768,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_813</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -26423,12 +26778,12 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -26530,12 +26885,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -26570,7 +26925,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_811</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -26580,12 +26935,12 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -26687,12 +27042,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -26727,7 +27082,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_811</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -26737,12 +27092,12 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -26844,12 +27199,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -26884,7 +27239,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_781</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -26894,12 +27249,12 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -27001,12 +27356,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -27041,7 +27396,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_815</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -27051,12 +27406,12 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -27158,12 +27513,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -27198,7 +27553,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_789</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -27208,12 +27563,12 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -27315,12 +27670,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -27355,7 +27710,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_790</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -27365,12 +27720,12 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -27472,12 +27827,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -27512,7 +27867,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_791</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -27522,12 +27877,12 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -27629,12 +27984,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -27669,7 +28024,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_791</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -27679,12 +28034,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -27786,12 +28141,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -27826,7 +28181,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_793</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -27836,12 +28191,12 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -27943,12 +28298,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -27983,7 +28338,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_793</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -27993,12 +28348,12 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -28100,12 +28455,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -28140,7 +28495,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_783</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -28150,12 +28505,12 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -28257,12 +28612,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -28297,7 +28652,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_784</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -28307,12 +28662,12 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -28414,12 +28769,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module, Statement, HIERARCHY</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -28454,7 +28809,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_785</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -28464,12 +28819,12 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -28571,12 +28926,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module, Statement, HIERARCHY</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -28611,7 +28966,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_785</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -28621,12 +28976,12 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -28728,12 +29083,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -28768,7 +29123,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_798</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -28778,12 +29133,12 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -28885,12 +29240,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -28925,7 +29280,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_802</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -28935,12 +29290,12 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -29042,12 +29397,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -29082,7 +29437,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_799</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -29092,12 +29447,12 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -29199,12 +29554,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -29239,7 +29594,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_800</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -29249,12 +29604,12 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -29356,12 +29711,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -29396,7 +29751,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_801</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -29406,12 +29761,12 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -29513,12 +29868,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -29553,7 +29908,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_803</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -29563,12 +29918,12 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -29670,12 +30025,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -29710,7 +30065,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_772</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -29720,12 +30075,12 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -29827,12 +30182,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -29867,7 +30222,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_773</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -29877,12 +30232,12 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -29984,12 +30339,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -30024,7 +30379,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_774</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -30034,12 +30389,12 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -30141,12 +30496,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -30181,7 +30536,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_775</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -30191,12 +30546,12 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -30298,12 +30653,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -30338,7 +30693,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_776</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -30348,12 +30703,12 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -30455,12 +30810,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -30495,7 +30850,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_777</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -30505,12 +30860,12 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -30612,12 +30967,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -30652,7 +31007,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_778</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -30662,12 +31017,12 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -30769,12 +31124,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -30809,7 +31164,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_779</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -30819,12 +31174,12 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -30926,12 +31281,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -30966,7 +31321,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_780</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -30976,12 +31331,12 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -31083,12 +31438,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -31123,7 +31478,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_806</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -31133,12 +31488,12 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -31240,12 +31595,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -31280,7 +31635,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_807</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -31290,12 +31645,12 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -31397,12 +31752,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -31437,7 +31792,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_816</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -31447,12 +31802,12 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -31554,12 +31909,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -31594,7 +31949,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_817</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -31604,12 +31959,12 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -31711,12 +32066,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -31751,7 +32106,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_818</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -31761,12 +32116,12 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -31868,12 +32223,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -31908,7 +32263,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_819</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -31918,12 +32273,12 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -32025,12 +32380,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -32065,7 +32420,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_820</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -32075,12 +32430,12 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -32182,12 +32537,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -32222,7 +32577,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_821</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -32232,12 +32587,12 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -32339,12 +32694,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -32379,7 +32734,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_822</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -32389,12 +32744,12 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -32496,12 +32851,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -32536,7 +32891,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_823</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -32546,12 +32901,12 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -32653,12 +33008,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -32693,7 +33048,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_824</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -32703,12 +33058,12 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -32810,12 +33165,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -32850,7 +33205,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_826</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -32860,12 +33215,12 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -32967,12 +33322,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -33007,7 +33362,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_827</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -33017,12 +33372,12 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -33124,12 +33479,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -33164,7 +33519,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_828</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -33174,12 +33529,12 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
@@ -33281,12 +33636,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -33321,7 +33676,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_829</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -33331,12 +33686,12 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -33438,12 +33793,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -33478,7 +33833,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_825</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -33488,12 +33843,12 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -33595,12 +33950,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -33635,7 +33990,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_839</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -33645,12 +34000,12 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -33752,12 +34107,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -33792,7 +34147,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_840</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -33802,12 +34157,12 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -33909,12 +34264,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -33949,7 +34304,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_841</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -33959,12 +34314,12 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -34066,12 +34421,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -34106,7 +34461,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_835</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -34116,12 +34471,12 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -34223,12 +34578,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -34263,7 +34618,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_836</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -34273,12 +34628,12 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -34380,12 +34735,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">AUTO</t>
+          <t xml:space="preserve">FIELDS</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Goal, Module=AESDMA_RD_DESC, Statement=n_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] = r_rdAddr[AXI_ADDR_WD-1:ADDR_BASE_LSB] + {{(AXI_ADDR_WD-ADDR_BASE_LSB-AXI_LEN_WD){1'b0}}, w_rdBurstLen} + 1;, HIERARCHY=:BOS_AESDMA:u_AESDMA_TOP@AESDMA_TOP_DCLS:u_aesdma_top@AESDMA_TOP:u_AESDMA_RD_DESC@AESDMA_RD_DESC</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -34420,7 +34775,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t xml:space="preserve">W164a_837</t>
+          <t xml:space="preserve">W164a_808</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -34430,12 +34785,12 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">pnson</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">

</xml_diff>